<commit_message>
ready to set up
</commit_message>
<xml_diff>
--- a/LinMeas/Fiber2/ITest2/Results.xlsx
+++ b/LinMeas/Fiber2/ITest2/Results.xlsx
@@ -1,31 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Diego\git\6s7p\LinMeas\Fiber2\Intentsity test\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Wolfwalker\Documents\git\6s7p\LinMeas\Fiber2\ITest2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D15545E-46C8-4A86-B8E2-493B6942092C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDE122DB-C2A0-4AFA-B6AF-383B910CE371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="temp" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">Sheet1!$B$3:$B$12</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">Sheet1!$C$3:$C$12</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">Sheet1!$E$3:$E$11</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">Sheet1!$F$3:$F$11</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">Sheet1!$H$3:$H$13</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">Sheet1!$I$3:$I$13</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">Sheet1!$L$3:$L$5</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">Sheet1!$M$3:$M$5</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -40,15 +30,12 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="5">
   <si>
     <t>Low</t>
   </si>
@@ -228,12 +215,6 @@
                 <c:pt idx="8">
                   <c:v>9</c:v>
                 </c:pt>
-                <c:pt idx="9">
-                  <c:v>10</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>11</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -244,34 +225,31 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>4.7712876792141902E-2</c:v>
+                  <c:v>0.13538022852761</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.8164394607539802E-2</c:v>
+                  <c:v>0.13465177191208699</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.6841778247040701E-2</c:v>
+                  <c:v>0.13481086685298899</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.7930772270805097E-2</c:v>
+                  <c:v>0.13540718732719201</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4.7916464907701899E-2</c:v>
+                  <c:v>0.13459217279489799</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4.8260922216410498E-2</c:v>
+                  <c:v>0.134594471980475</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>4.78940969094463E-2</c:v>
+                  <c:v>0.13522025484822101</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4.8596600010608303E-2</c:v>
+                  <c:v>0.13586271616981099</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>4.8529352775302501E-2</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>4.7865665132403999E-2</c:v>
+                  <c:v>0.135030590966186</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -341,12 +319,6 @@
                 <c:pt idx="8">
                   <c:v>9</c:v>
                 </c:pt>
-                <c:pt idx="9">
-                  <c:v>10</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>11</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -357,31 +329,31 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>4.64988576797742E-2</c:v>
+                  <c:v>0.13518210250875301</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.6994016686578502E-2</c:v>
+                  <c:v>0.13518946121606501</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.6706160693399598E-2</c:v>
+                  <c:v>0.136375992114487</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.7411507849964798E-2</c:v>
+                  <c:v>0.13555559802936601</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4.7895126407649001E-2</c:v>
+                  <c:v>0.13620731346533299</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4.7913746274083902E-2</c:v>
+                  <c:v>0.13588543565528499</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>4.7278928857606699E-2</c:v>
+                  <c:v>0.13482343117842499</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4.8060993633046702E-2</c:v>
+                  <c:v>0.136797430096464</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>4.7564085785623399E-2</c:v>
+                  <c:v>0.136285928993195</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -451,12 +423,6 @@
                 <c:pt idx="8">
                   <c:v>9</c:v>
                 </c:pt>
-                <c:pt idx="9">
-                  <c:v>10</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>11</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -467,37 +433,31 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>4.7594086855872998E-2</c:v>
+                  <c:v>0.13548958029595701</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.7865832680007402E-2</c:v>
+                  <c:v>0.13535257602050901</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.7946198533546001E-2</c:v>
+                  <c:v>0.13521437182562601</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.7958321334516898E-2</c:v>
+                  <c:v>0.13547579777680199</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4.7745472800668702E-2</c:v>
+                  <c:v>0.135355456711137</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4.7683759372150601E-2</c:v>
+                  <c:v>0.13562845171119001</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>4.79771761493403E-2</c:v>
+                  <c:v>0.135063967225622</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4.7459600367847798E-2</c:v>
+                  <c:v>0.13488752919092301</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>4.7677254085627299E-2</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>4.79891735986843E-2</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>4.7740785482986298E-2</c:v>
+                  <c:v>0.13488940608340499</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -685,6 +645,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -692,7 +653,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -812,34 +772,31 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>0.14650866185077294</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.14650866185077294</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.14650866185077294</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.14650866185077294</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.14650866185077294</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.14650866185077294</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.14650866185077294</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.14650866185077294</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.14650866185077294</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0.14650866185077294</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -851,34 +808,31 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>4.7712876792141902E-2</c:v>
+                  <c:v>0.13538022852761</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.8164394607539802E-2</c:v>
+                  <c:v>0.13465177191208699</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.6841778247040701E-2</c:v>
+                  <c:v>0.13481086685298899</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.7930772270805097E-2</c:v>
+                  <c:v>0.13540718732719201</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4.7916464907701899E-2</c:v>
+                  <c:v>0.13459217279489799</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4.8260922216410498E-2</c:v>
+                  <c:v>0.134594471980475</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>4.78940969094463E-2</c:v>
+                  <c:v>0.13522025484822101</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4.8596600010608303E-2</c:v>
+                  <c:v>0.13586271616981099</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>4.8529352775302501E-2</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>4.7865665132403999E-2</c:v>
+                  <c:v>0.135030590966186</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -925,31 +879,31 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>0.38314167044465475</c:v>
+                  <c:v>0.43</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.38314167044465475</c:v>
+                  <c:v>0.43</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.38314167044465475</c:v>
+                  <c:v>0.43</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.38314167044465475</c:v>
+                  <c:v>0.43</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.38314167044465475</c:v>
+                  <c:v>0.43</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.38314167044465475</c:v>
+                  <c:v>0.43</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.38314167044465475</c:v>
+                  <c:v>0.43</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.38314167044465475</c:v>
+                  <c:v>0.43</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.38314167044465475</c:v>
+                  <c:v>0.43</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -961,31 +915,31 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>4.64988576797742E-2</c:v>
+                  <c:v>0.13518210250875301</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.6994016686578502E-2</c:v>
+                  <c:v>0.13518946121606501</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.6706160693399598E-2</c:v>
+                  <c:v>0.136375992114487</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.7411507849964798E-2</c:v>
+                  <c:v>0.13555559802936601</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4.7895126407649001E-2</c:v>
+                  <c:v>0.13620731346533299</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4.7913746274083902E-2</c:v>
+                  <c:v>0.13588543565528499</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>4.7278928857606699E-2</c:v>
+                  <c:v>0.13482343117842499</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4.8060993633046702E-2</c:v>
+                  <c:v>0.136797430096464</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>4.7564085785623399E-2</c:v>
+                  <c:v>0.136285928993195</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1032,37 +986,31 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>1.0142937182713132</c:v>
+                  <c:v>1.9</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.0142937182713132</c:v>
+                  <c:v>1.9</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.0142937182713132</c:v>
+                  <c:v>1.9</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.0142937182713132</c:v>
+                  <c:v>1.9</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.0142937182713132</c:v>
+                  <c:v>1.9</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.0142937182713132</c:v>
+                  <c:v>1.9</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.0142937182713132</c:v>
+                  <c:v>1.9</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.0142937182713132</c:v>
+                  <c:v>1.9</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.0142937182713132</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>1.0142937182713132</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>1.0142937182713132</c:v>
+                  <c:v>1.9</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1074,37 +1022,31 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>4.7594086855872998E-2</c:v>
+                  <c:v>0.13548958029595701</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.7865832680007402E-2</c:v>
+                  <c:v>0.13535257602050901</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.7946198533546001E-2</c:v>
+                  <c:v>0.13521437182562601</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.7958321334516898E-2</c:v>
+                  <c:v>0.13547579777680199</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4.7745472800668702E-2</c:v>
+                  <c:v>0.135355456711137</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4.7683759372150601E-2</c:v>
+                  <c:v>0.13562845171119001</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>4.79771761493403E-2</c:v>
+                  <c:v>0.135063967225622</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4.7459600367847798E-2</c:v>
+                  <c:v>0.13488752919092301</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>4.7677254085627299E-2</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>4.79891735986843E-2</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>4.7740785482986298E-2</c:v>
+                  <c:v>0.13488940608340499</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1151,13 +1093,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>0.19650866185077293</c:v>
+                  <c:v>0.25</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.43314167044465474</c:v>
+                  <c:v>0.48</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.0642937182713132</c:v>
+                  <c:v>1.95</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1169,13 +1111,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>4.7971292386940097E-2</c:v>
+                  <c:v>0.13506114015327431</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.736926931863631E-2</c:v>
+                  <c:v>0.13581141036193034</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.7785241932840776E-2</c:v>
+                  <c:v>0.13526190409346342</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1332,6 +1274,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1339,7 +1282,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1520,13 +1462,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>0.19650866185077293</c:v>
+                  <c:v>0.25</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.43314167044465474</c:v>
+                  <c:v>0.48</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.0642937182713132</c:v>
+                  <c:v>1.95</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1538,13 +1480,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>4.7971292386940097E-2</c:v>
+                  <c:v>0.13506114015327431</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.736926931863631E-2</c:v>
+                  <c:v>0.13581141036193034</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.7785241932840776E-2</c:v>
+                  <c:v>0.13526190409346342</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1701,6 +1643,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1708,7 +1651,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1758,6 +1700,35 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Low</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> Absorption</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -2119,6 +2090,66 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>PD</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> Volt</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -2181,6 +2212,61 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>ABs Coeff</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -2232,6 +2318,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2239,7 +2326,664 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>High</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> Absorption</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="3.7502187226596674E-3"/>
+                  <c:y val="-0.46035250801983085"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$V$9:$V$36</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="28"/>
+                <c:pt idx="0">
+                  <c:v>0.2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.43</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.43</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.43</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.43</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.43</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.43</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.43</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.43</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.43</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1.9</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1.9</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1.9</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>1.9</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>1.9</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>1.9</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>1.9</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>1.9</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>1.9</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$W$9:$W$36</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="28"/>
+                <c:pt idx="0">
+                  <c:v>0.13538022852761</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.13465177191208699</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.13481086685298899</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.13540718732719201</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.13459217279489799</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.134594471980475</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.13522025484822101</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.13586271616981099</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.135030590966186</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.13518210250875301</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.13518946121606501</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.136375992114487</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.13555559802936601</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.13620731346533299</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.13588543565528499</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.13482343117842499</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.136797430096464</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.136285928993195</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.13548958029595701</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.13535257602050901</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.13521437182562601</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.13547579777680199</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.135355456711137</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.13562845171119001</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.135063967225622</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.13488752919092301</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0.13488940608340499</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-03F6-4FE2-98D3-3C48569ECBA6}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1160170912"/>
+        <c:axId val="1160171392"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1160170912"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>PD Volt</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1160171392"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1160171392"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Abs</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> Coeff</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1160170912"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2434,6 +3178,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -3983,6 +4767,522 @@
 </file>
 
 <file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -4503,15 +5803,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>152400</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:colOff>520700</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>533400</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>9523</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>292100</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>41273</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4574,16 +5874,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>571500</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>82550</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>174625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>22</xdr:col>
-      <xdr:colOff>390525</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>185737</xdr:rowOff>
+      <xdr:col>38</xdr:col>
+      <xdr:colOff>320675</xdr:colOff>
+      <xdr:row>60</xdr:row>
+      <xdr:rowOff>52387</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4610,16 +5910,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>347662</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>100012</xdr:rowOff>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>17462</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>23812</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>42862</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>176212</xdr:rowOff>
+      <xdr:col>36</xdr:col>
+      <xdr:colOff>322262</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>100012</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4639,6 +5939,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>377825</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>12700</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>73025</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>177800</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="9" name="Chart 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{94CAF1DA-E611-D2BE-1969-DADBCB7A2304}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -4910,13 +6246,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T38"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AI38"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="15" max="15" width="14.7109375" customWidth="1"/>
+    <col min="15" max="15" width="14.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -4927,9 +6263,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="B2">
-        <v>0.14650866185077294</v>
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="B2" s="1">
+        <v>0.2</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>3</v>
@@ -4937,8 +6273,8 @@
       <c r="D2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E2">
-        <v>0.38314167044465475</v>
+      <c r="E2" s="1">
+        <v>0.43</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>3</v>
@@ -4947,7 +6283,7 @@
         <v>4</v>
       </c>
       <c r="H2">
-        <v>1.0142937182713132</v>
+        <v>1.9</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>3</v>
@@ -4955,297 +6291,414 @@
       <c r="J2" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="AD2">
+        <v>1</v>
+      </c>
+      <c r="AF2">
+        <v>2</v>
+      </c>
+      <c r="AH2">
+        <v>3</v>
+      </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1</v>
       </c>
-      <c r="B3">
-        <v>0.14650866185077294</v>
+      <c r="B3" s="1">
+        <v>0.2</v>
       </c>
       <c r="C3" s="1">
-        <v>4.7712876792141902E-2</v>
+        <v>0.13538022852761</v>
       </c>
       <c r="D3" s="1">
-        <v>3.5448009376697902</v>
-      </c>
-      <c r="E3">
-        <v>0.38314167044465475</v>
+        <v>0.83823758715430297</v>
+      </c>
+      <c r="E3" s="1">
+        <v>0.43</v>
       </c>
       <c r="F3" s="1">
-        <v>4.64988576797742E-2</v>
+        <v>0.13518210250875301</v>
       </c>
       <c r="G3" s="1">
-        <v>3.5665516980494898</v>
+        <v>0.85033107985282597</v>
       </c>
       <c r="H3">
-        <v>1.0142937182713132</v>
+        <v>1.9</v>
       </c>
       <c r="I3" s="1">
-        <v>4.7594086855872998E-2</v>
+        <v>0.13548958029595701</v>
       </c>
       <c r="J3" s="1">
-        <v>3.5961295088708498</v>
+        <v>0.87131792083959003</v>
       </c>
       <c r="L3">
         <f>B2+0.05</f>
-        <v>0.19650866185077293</v>
+        <v>0.25</v>
       </c>
       <c r="M3">
         <f>AVERAGE(C3:C13)</f>
-        <v>4.7971292386940097E-2</v>
+        <v>0.13506114015327431</v>
       </c>
       <c r="N3">
         <f>_xlfn.STDEV.S(C3:C12)</f>
-        <v>4.9305847408479984E-4</v>
+        <v>4.4134305462615887E-4</v>
       </c>
       <c r="O3">
         <f>N3/SQRT(COUNT(C3:C12))</f>
-        <v>1.5591877977550722E-4</v>
+        <v>1.4711435154205296E-4</v>
       </c>
       <c r="P3">
         <f>O3/M3</f>
-        <v>3.250251807223672E-3</v>
+        <v>1.0892426302273181E-3</v>
+      </c>
+      <c r="AD3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="AE3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="AF3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="AG3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="AH3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="AI3" s="1" t="s">
+        <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2</v>
       </c>
-      <c r="B4">
-        <v>0.14650866185077294</v>
+      <c r="B4" s="1">
+        <v>0.2</v>
       </c>
       <c r="C4" s="1">
-        <v>4.8164394607539802E-2</v>
+        <v>0.13465177191208699</v>
       </c>
       <c r="D4" s="1">
-        <v>3.5357963224140998</v>
-      </c>
-      <c r="E4">
-        <v>0.38314167044465475</v>
+        <v>0.83919127498099999</v>
+      </c>
+      <c r="E4" s="1">
+        <v>0.43</v>
       </c>
       <c r="F4" s="1">
-        <v>4.6994016686578502E-2</v>
+        <v>0.13518946121606501</v>
       </c>
       <c r="G4" s="1">
-        <v>3.5673410121687499</v>
+        <v>0.85015059059048204</v>
       </c>
       <c r="H4">
-        <v>1.0142937182713132</v>
+        <v>1.9</v>
       </c>
       <c r="I4" s="1">
-        <v>4.7865832680007402E-2</v>
+        <v>0.13535257602050901</v>
       </c>
       <c r="J4" s="1">
-        <v>3.59249324983996</v>
+        <v>0.87199124996167299</v>
       </c>
       <c r="L4">
         <f>E3+0.05</f>
-        <v>0.43314167044465474</v>
+        <v>0.48</v>
       </c>
       <c r="M4">
         <f>AVERAGE(F3:F13)</f>
-        <v>4.736926931863631E-2</v>
+        <v>0.13581141036193034</v>
       </c>
       <c r="N4">
         <f>_xlfn.STDEV.S(F3:F12)</f>
-        <v>5.5198576932045159E-4</v>
+        <v>6.6169917122627727E-4</v>
       </c>
       <c r="O4">
         <f>N4/SQRT(COUNT(F3:F12))</f>
-        <v>1.8399525644015053E-4</v>
+        <v>2.2056639040875909E-4</v>
       </c>
       <c r="P4">
         <f t="shared" ref="P4:P5" si="0">O4/M4</f>
-        <v>3.8842747436630184E-3</v>
+        <v>1.6240637647526165E-3</v>
+      </c>
+      <c r="AD4" s="1">
+        <v>0.13538022852761</v>
+      </c>
+      <c r="AE4" s="1">
+        <v>0.83823758715430297</v>
+      </c>
+      <c r="AF4" s="1">
+        <v>0.13518210250875301</v>
+      </c>
+      <c r="AG4" s="1">
+        <v>0.85033107985282597</v>
+      </c>
+      <c r="AH4" s="1">
+        <v>0.13548958029595701</v>
+      </c>
+      <c r="AI4" s="1">
+        <v>0.87131792083959003</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>3</v>
       </c>
-      <c r="B5">
-        <v>0.14650866185077294</v>
+      <c r="B5" s="1">
+        <v>0.2</v>
       </c>
       <c r="C5" s="1">
-        <v>4.6841778247040701E-2</v>
+        <v>0.13481086685298899</v>
       </c>
       <c r="D5" s="1">
-        <v>3.5418406755249698</v>
-      </c>
-      <c r="E5">
-        <v>0.38314167044465475</v>
+        <v>0.83884357019737499</v>
+      </c>
+      <c r="E5" s="1">
+        <v>0.43</v>
       </c>
       <c r="F5" s="1">
-        <v>4.6706160693399598E-2</v>
+        <v>0.136375992114487</v>
       </c>
       <c r="G5" s="1">
-        <v>3.5667619989188299</v>
+        <v>0.85094968351988898</v>
       </c>
       <c r="H5">
-        <v>1.0142937182713132</v>
+        <v>1.9</v>
       </c>
       <c r="I5" s="1">
-        <v>4.7946198533546001E-2</v>
+        <v>0.13521437182562601</v>
       </c>
       <c r="J5" s="1">
-        <v>3.5944805290050401</v>
+        <v>0.87225000855282098</v>
       </c>
       <c r="L5">
         <f>H3+0.05</f>
-        <v>1.0642937182713132</v>
+        <v>1.95</v>
       </c>
       <c r="M5">
         <f>AVERAGE(I3:I13)</f>
-        <v>4.7785241932840776E-2</v>
+        <v>0.13526190409346342</v>
       </c>
       <c r="N5">
         <f>_xlfn.STDEV.S(I3:I13)</f>
-        <v>1.757515235496052E-4</v>
+        <v>2.6675533334150238E-4</v>
       </c>
       <c r="O5">
         <f>N5/SQRT(COUNT(I3:I13))</f>
-        <v>5.2991078177031954E-5</v>
+        <v>8.8918444447167456E-5</v>
       </c>
       <c r="P5">
         <f t="shared" si="0"/>
-        <v>1.1089423435693318E-3</v>
+        <v>6.5737980729390364E-4</v>
+      </c>
+      <c r="AD5" s="1">
+        <v>0.13465177191208699</v>
+      </c>
+      <c r="AE5" s="1">
+        <v>0.83919127498099999</v>
+      </c>
+      <c r="AF5" s="1">
+        <v>0.13518946121606501</v>
+      </c>
+      <c r="AG5" s="1">
+        <v>0.85015059059048204</v>
+      </c>
+      <c r="AH5" s="1">
+        <v>0.13535257602050901</v>
+      </c>
+      <c r="AI5" s="1">
+        <v>0.87199124996167299</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>4</v>
       </c>
-      <c r="B6">
-        <v>0.14650866185077294</v>
+      <c r="B6" s="1">
+        <v>0.2</v>
       </c>
       <c r="C6" s="1">
-        <v>4.7930772270805097E-2</v>
+        <v>0.13540718732719201</v>
       </c>
       <c r="D6" s="1">
-        <v>3.5417194207225</v>
-      </c>
-      <c r="E6">
-        <v>0.38314167044465475</v>
+        <v>0.83875717395846305</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0.43</v>
       </c>
       <c r="F6" s="1">
-        <v>4.7411507849964798E-2</v>
+        <v>0.13555559802936601</v>
       </c>
       <c r="G6" s="1">
-        <v>3.56094145962558</v>
+        <v>0.85058451946696201</v>
       </c>
       <c r="H6">
-        <v>1.0142937182713132</v>
+        <v>1.9</v>
       </c>
       <c r="I6" s="1">
-        <v>4.7958321334516898E-2</v>
+        <v>0.13547579777680199</v>
       </c>
       <c r="J6" s="1">
-        <v>3.5940387704001302</v>
+        <v>0.87247757181119401</v>
       </c>
       <c r="R6">
         <f>AVERAGE(M3:M5)</f>
-        <v>4.7708601212805728E-2</v>
+        <v>0.13537815153622268</v>
       </c>
       <c r="S6">
         <f>0.00003/R6</f>
-        <v>6.2881742992598017E-4</v>
+        <v>2.2160148930658874E-4</v>
+      </c>
+      <c r="AD6" s="1">
+        <v>0.13481086685298899</v>
+      </c>
+      <c r="AE6" s="1">
+        <v>0.83884357019737499</v>
+      </c>
+      <c r="AF6" s="1">
+        <v>0.136375992114487</v>
+      </c>
+      <c r="AG6" s="1">
+        <v>0.85094968351988898</v>
+      </c>
+      <c r="AH6" s="1">
+        <v>0.13521437182562601</v>
+      </c>
+      <c r="AI6" s="1">
+        <v>0.87225000855282098</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>5</v>
       </c>
-      <c r="B7">
-        <v>0.14650866185077294</v>
+      <c r="B7" s="1">
+        <v>0.2</v>
       </c>
       <c r="C7" s="1">
-        <v>4.7916464907701899E-2</v>
+        <v>0.13459217279489799</v>
       </c>
       <c r="D7" s="1">
-        <v>3.5378767865990901</v>
-      </c>
-      <c r="E7">
-        <v>0.38314167044465475</v>
+        <v>0.83882303502512201</v>
+      </c>
+      <c r="E7" s="1">
+        <v>0.43</v>
       </c>
       <c r="F7" s="1">
-        <v>4.7895126407649001E-2</v>
+        <v>0.13620731346533299</v>
       </c>
       <c r="G7" s="1">
-        <v>3.56206709895842</v>
+        <v>0.851139563886669</v>
       </c>
       <c r="H7">
-        <v>1.0142937182713132</v>
+        <v>1.9</v>
       </c>
       <c r="I7" s="1">
-        <v>4.7745472800668702E-2</v>
+        <v>0.135355456711137</v>
       </c>
       <c r="J7" s="1">
-        <v>3.5936279138245402</v>
+        <v>0.87673491688351202</v>
+      </c>
+      <c r="AD7" s="1">
+        <v>0.13540718732719201</v>
+      </c>
+      <c r="AE7" s="1">
+        <v>0.83875717395846305</v>
+      </c>
+      <c r="AF7" s="1">
+        <v>0.13555559802936601</v>
+      </c>
+      <c r="AG7" s="1">
+        <v>0.85058451946696201</v>
+      </c>
+      <c r="AH7" s="1">
+        <v>0.13547579777680199</v>
+      </c>
+      <c r="AI7" s="1">
+        <v>0.87247757181119401</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>6</v>
       </c>
-      <c r="B8">
-        <v>0.14650866185077294</v>
+      <c r="B8" s="1">
+        <v>0.2</v>
       </c>
       <c r="C8" s="1">
-        <v>4.8260922216410498E-2</v>
+        <v>0.134594471980475</v>
       </c>
       <c r="D8" s="1">
-        <v>3.5414868387468101</v>
-      </c>
-      <c r="E8">
-        <v>0.38314167044465475</v>
+        <v>0.83840915587926101</v>
+      </c>
+      <c r="E8" s="1">
+        <v>0.43</v>
       </c>
       <c r="F8" s="1">
-        <v>4.7913746274083902E-2</v>
+        <v>0.13588543565528499</v>
       </c>
       <c r="G8" s="1">
-        <v>3.5623345096529202</v>
+        <v>0.85115781595748696</v>
       </c>
       <c r="H8">
-        <v>1.0142937182713132</v>
+        <v>1.9</v>
       </c>
       <c r="I8" s="1">
-        <v>4.7683759372150601E-2</v>
+        <v>0.13562845171119001</v>
       </c>
       <c r="J8" s="1">
-        <v>3.5944944602968598</v>
+        <v>0.87671353645148498</v>
+      </c>
+      <c r="AD8" s="1">
+        <v>0.13459217279489799</v>
+      </c>
+      <c r="AE8" s="1">
+        <v>0.83882303502512201</v>
+      </c>
+      <c r="AF8" s="1">
+        <v>0.13620731346533299</v>
+      </c>
+      <c r="AG8" s="1">
+        <v>0.851139563886669</v>
+      </c>
+      <c r="AH8" s="1">
+        <v>0.135355456711137</v>
+      </c>
+      <c r="AI8" s="1">
+        <v>0.87673491688351202</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>7</v>
       </c>
-      <c r="B9">
-        <v>0.14650866185077294</v>
+      <c r="B9" s="1">
+        <v>0.2</v>
       </c>
       <c r="C9" s="1">
-        <v>4.78940969094463E-2</v>
+        <v>0.13522025484822101</v>
       </c>
       <c r="D9" s="1">
-        <v>3.5478707328833998</v>
-      </c>
-      <c r="E9">
-        <v>0.38314167044465475</v>
+        <v>0.83712407596487803</v>
+      </c>
+      <c r="E9" s="1">
+        <v>0.43</v>
       </c>
       <c r="F9" s="1">
-        <v>4.7278928857606699E-2</v>
+        <v>0.13482343117842499</v>
       </c>
       <c r="G9" s="1">
-        <v>3.5657460976611</v>
+        <v>0.85158332958003902</v>
       </c>
       <c r="H9">
-        <v>1.0142937182713132</v>
+        <v>1.9</v>
       </c>
       <c r="I9" s="1">
-        <v>4.79771761493403E-2</v>
+        <v>0.135063967225622</v>
       </c>
       <c r="J9" s="1">
-        <v>3.5943638050046101</v>
+        <v>0.87668269721274505</v>
       </c>
       <c r="S9">
         <v>0.14650866185077294</v>
@@ -5253,37 +6706,61 @@
       <c r="T9" s="1">
         <v>4.7712876792141902E-2</v>
       </c>
+      <c r="V9" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="W9" s="1">
+        <v>0.13538022852761</v>
+      </c>
+      <c r="AD9" s="1">
+        <v>0.134594471980475</v>
+      </c>
+      <c r="AE9" s="1">
+        <v>0.83840915587926101</v>
+      </c>
+      <c r="AF9" s="1">
+        <v>0.13588543565528499</v>
+      </c>
+      <c r="AG9" s="1">
+        <v>0.85115781595748696</v>
+      </c>
+      <c r="AH9" s="1">
+        <v>0.13562845171119001</v>
+      </c>
+      <c r="AI9" s="1">
+        <v>0.87671353645148498</v>
+      </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>8</v>
       </c>
-      <c r="B10">
-        <v>0.14650866185077294</v>
+      <c r="B10" s="1">
+        <v>0.2</v>
       </c>
       <c r="C10" s="1">
-        <v>4.8596600010608303E-2</v>
+        <v>0.13586271616981099</v>
       </c>
       <c r="D10" s="1">
-        <v>3.5466910309338102</v>
-      </c>
-      <c r="E10">
-        <v>0.38314167044465475</v>
+        <v>0.84038736827086302</v>
+      </c>
+      <c r="E10" s="1">
+        <v>0.43</v>
       </c>
       <c r="F10" s="1">
-        <v>4.8060993633046702E-2</v>
+        <v>0.136797430096464</v>
       </c>
       <c r="G10" s="1">
-        <v>3.5668519079769898</v>
+        <v>0.85055175627919799</v>
       </c>
       <c r="H10">
-        <v>1.0142937182713132</v>
+        <v>1.9</v>
       </c>
       <c r="I10" s="1">
-        <v>4.7459600367847798E-2</v>
+        <v>0.13488752919092301</v>
       </c>
       <c r="J10" s="1">
-        <v>3.59270769294542</v>
+        <v>0.87699702135039803</v>
       </c>
       <c r="S10">
         <v>0.14650866185077294</v>
@@ -5291,37 +6768,61 @@
       <c r="T10" s="1">
         <v>4.8164394607539802E-2</v>
       </c>
+      <c r="V10" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="W10" s="1">
+        <v>0.13465177191208699</v>
+      </c>
+      <c r="AD10" s="1">
+        <v>0.13522025484822101</v>
+      </c>
+      <c r="AE10" s="1">
+        <v>0.83712407596487803</v>
+      </c>
+      <c r="AF10" s="1">
+        <v>0.13482343117842499</v>
+      </c>
+      <c r="AG10" s="1">
+        <v>0.85158332958003902</v>
+      </c>
+      <c r="AH10" s="1">
+        <v>0.135063967225622</v>
+      </c>
+      <c r="AI10" s="1">
+        <v>0.87668269721274505</v>
+      </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>9</v>
       </c>
-      <c r="B11">
-        <v>0.14650866185077294</v>
+      <c r="B11" s="1">
+        <v>0.2</v>
       </c>
       <c r="C11" s="1">
-        <v>4.8529352775302501E-2</v>
+        <v>0.135030590966186</v>
       </c>
       <c r="D11" s="1">
-        <v>3.5437420973704699</v>
-      </c>
-      <c r="E11">
-        <v>0.38314167044465475</v>
+        <v>0.83899664790976702</v>
+      </c>
+      <c r="E11" s="1">
+        <v>0.43</v>
       </c>
       <c r="F11" s="1">
-        <v>4.7564085785623399E-2</v>
+        <v>0.136285928993195</v>
       </c>
       <c r="G11" s="1">
-        <v>3.56326684995501</v>
+        <v>0.85090465377646096</v>
       </c>
       <c r="H11">
-        <v>1.0142937182713132</v>
+        <v>1.9</v>
       </c>
       <c r="I11" s="1">
-        <v>4.7677254085627299E-2</v>
+        <v>0.13488940608340499</v>
       </c>
       <c r="J11" s="1">
-        <v>3.5932752329519602</v>
+        <v>0.87686535046181002</v>
       </c>
       <c r="S11">
         <v>0.14650866185077294</v>
@@ -5329,233 +6830,409 @@
       <c r="T11" s="1">
         <v>4.6841778247040701E-2</v>
       </c>
+      <c r="V11" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="W11" s="1">
+        <v>0.13481086685298899</v>
+      </c>
+      <c r="AD11" s="1">
+        <v>0.13586271616981099</v>
+      </c>
+      <c r="AE11" s="1">
+        <v>0.84038736827086302</v>
+      </c>
+      <c r="AF11" s="1">
+        <v>0.136797430096464</v>
+      </c>
+      <c r="AG11" s="1">
+        <v>0.85055175627919799</v>
+      </c>
+      <c r="AH11" s="1">
+        <v>0.13488752919092301</v>
+      </c>
+      <c r="AI11" s="1">
+        <v>0.87699702135039803</v>
+      </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>10</v>
-      </c>
-      <c r="B12">
-        <v>0.14650866185077294</v>
-      </c>
-      <c r="C12" s="1">
-        <v>4.7865665132403999E-2</v>
-      </c>
-      <c r="D12" s="1">
-        <v>3.54315176654312</v>
-      </c>
-      <c r="H12">
-        <v>1.0142937182713132</v>
-      </c>
-      <c r="I12" s="1">
-        <v>4.79891735986843E-2</v>
-      </c>
-      <c r="J12" s="1">
-        <v>3.5930551102784101</v>
-      </c>
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
       <c r="S12">
         <v>0.14650866185077294</v>
       </c>
       <c r="T12" s="1">
         <v>4.7930772270805097E-2</v>
       </c>
+      <c r="V12" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="W12" s="1">
+        <v>0.13540718732719201</v>
+      </c>
+      <c r="AD12" s="1">
+        <v>0.135030590966186</v>
+      </c>
+      <c r="AE12" s="1">
+        <v>0.83899664790976702</v>
+      </c>
+      <c r="AF12" s="1">
+        <v>0.136285928993195</v>
+      </c>
+      <c r="AG12" s="1">
+        <v>0.85090465377646096</v>
+      </c>
+      <c r="AH12" s="1">
+        <v>0.13488940608340499</v>
+      </c>
+      <c r="AI12" s="1">
+        <v>0.87686535046181002</v>
+      </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>11</v>
-      </c>
-      <c r="H13">
-        <v>1.0142937182713132</v>
-      </c>
-      <c r="I13" s="1">
-        <v>4.7740785482986298E-2</v>
-      </c>
-      <c r="J13" s="1">
-        <v>3.5923112607248799</v>
-      </c>
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
       <c r="S13">
         <v>0.14650866185077294</v>
       </c>
       <c r="T13" s="1">
         <v>4.7916464907701899E-2</v>
       </c>
+      <c r="V13" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="W13" s="1">
+        <v>0.13459217279489799</v>
+      </c>
+      <c r="AF13" s="1">
+        <v>0.13638091085238799</v>
+      </c>
+      <c r="AG13" s="1">
+        <v>0.85101092318524996</v>
+      </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="S14">
         <v>0.14650866185077294</v>
       </c>
       <c r="T14" s="1">
         <v>4.8260922216410498E-2</v>
       </c>
+      <c r="V14" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="W14" s="1">
+        <v>0.134594471980475</v>
+      </c>
+      <c r="AF14" s="1">
+        <v>0.13648754807274699</v>
+      </c>
+      <c r="AG14" s="1">
+        <v>0.85154292457302105</v>
+      </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="S15">
         <v>0.14650866185077294</v>
       </c>
       <c r="T15" s="1">
         <v>4.78940969094463E-2</v>
       </c>
+      <c r="V15" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="W15" s="1">
+        <v>0.13522025484822101</v>
+      </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:35" x14ac:dyDescent="0.35">
       <c r="S16">
         <v>0.14650866185077294</v>
       </c>
       <c r="T16" s="1">
         <v>4.8596600010608303E-2</v>
       </c>
+      <c r="V16" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="W16" s="1">
+        <v>0.13586271616981099</v>
+      </c>
     </row>
-    <row r="17" spans="19:20" x14ac:dyDescent="0.25">
+    <row r="17" spans="19:23" x14ac:dyDescent="0.35">
       <c r="S17">
         <v>0.14650866185077294</v>
       </c>
       <c r="T17" s="1">
         <v>4.8529352775302501E-2</v>
       </c>
+      <c r="V17" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="W17" s="1">
+        <v>0.135030590966186</v>
+      </c>
     </row>
-    <row r="18" spans="19:20" x14ac:dyDescent="0.25">
+    <row r="18" spans="19:23" x14ac:dyDescent="0.35">
       <c r="S18">
         <v>0.14650866185077294</v>
       </c>
       <c r="T18" s="1">
         <v>4.7865665132403999E-2</v>
       </c>
+      <c r="V18" s="1">
+        <v>0.43</v>
+      </c>
+      <c r="W18" s="1">
+        <v>0.13518210250875301</v>
+      </c>
     </row>
-    <row r="19" spans="19:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="19:23" x14ac:dyDescent="0.35">
       <c r="S19">
         <v>0.38314167044465475</v>
       </c>
       <c r="T19" s="1">
         <v>4.64988576797742E-2</v>
       </c>
+      <c r="V19" s="1">
+        <v>0.43</v>
+      </c>
+      <c r="W19" s="1">
+        <v>0.13518946121606501</v>
+      </c>
     </row>
-    <row r="20" spans="19:20" x14ac:dyDescent="0.25">
+    <row r="20" spans="19:23" x14ac:dyDescent="0.35">
       <c r="S20">
         <v>0.38314167044465475</v>
       </c>
       <c r="T20" s="1">
         <v>4.6994016686578502E-2</v>
       </c>
+      <c r="V20" s="1">
+        <v>0.43</v>
+      </c>
+      <c r="W20" s="1">
+        <v>0.136375992114487</v>
+      </c>
     </row>
-    <row r="21" spans="19:20" x14ac:dyDescent="0.25">
+    <row r="21" spans="19:23" x14ac:dyDescent="0.35">
       <c r="S21">
         <v>0.38314167044465475</v>
       </c>
       <c r="T21" s="1">
         <v>4.6706160693399598E-2</v>
       </c>
+      <c r="V21" s="1">
+        <v>0.43</v>
+      </c>
+      <c r="W21" s="1">
+        <v>0.13555559802936601</v>
+      </c>
     </row>
-    <row r="22" spans="19:20" x14ac:dyDescent="0.25">
+    <row r="22" spans="19:23" x14ac:dyDescent="0.35">
       <c r="S22">
         <v>0.38314167044465475</v>
       </c>
       <c r="T22" s="1">
         <v>4.7411507849964798E-2</v>
       </c>
+      <c r="V22" s="1">
+        <v>0.43</v>
+      </c>
+      <c r="W22" s="1">
+        <v>0.13620731346533299</v>
+      </c>
     </row>
-    <row r="23" spans="19:20" x14ac:dyDescent="0.25">
+    <row r="23" spans="19:23" x14ac:dyDescent="0.35">
       <c r="S23">
         <v>0.38314167044465475</v>
       </c>
       <c r="T23" s="1">
         <v>4.7895126407649001E-2</v>
       </c>
+      <c r="V23" s="1">
+        <v>0.43</v>
+      </c>
+      <c r="W23" s="1">
+        <v>0.13588543565528499</v>
+      </c>
     </row>
-    <row r="24" spans="19:20" x14ac:dyDescent="0.25">
+    <row r="24" spans="19:23" x14ac:dyDescent="0.35">
       <c r="S24">
         <v>0.38314167044465475</v>
       </c>
       <c r="T24" s="1">
         <v>4.7913746274083902E-2</v>
       </c>
+      <c r="V24" s="1">
+        <v>0.43</v>
+      </c>
+      <c r="W24" s="1">
+        <v>0.13482343117842499</v>
+      </c>
     </row>
-    <row r="25" spans="19:20" x14ac:dyDescent="0.25">
+    <row r="25" spans="19:23" x14ac:dyDescent="0.35">
       <c r="S25">
         <v>0.38314167044465475</v>
       </c>
       <c r="T25" s="1">
         <v>4.7278928857606699E-2</v>
       </c>
+      <c r="V25" s="1">
+        <v>0.43</v>
+      </c>
+      <c r="W25" s="1">
+        <v>0.136797430096464</v>
+      </c>
     </row>
-    <row r="26" spans="19:20" x14ac:dyDescent="0.25">
+    <row r="26" spans="19:23" x14ac:dyDescent="0.35">
       <c r="S26">
         <v>0.38314167044465475</v>
       </c>
       <c r="T26" s="1">
         <v>4.8060993633046702E-2</v>
       </c>
+      <c r="V26" s="1">
+        <v>0.43</v>
+      </c>
+      <c r="W26" s="1">
+        <v>0.136285928993195</v>
+      </c>
     </row>
-    <row r="27" spans="19:20" x14ac:dyDescent="0.25">
+    <row r="27" spans="19:23" x14ac:dyDescent="0.35">
       <c r="S27">
         <v>0.38314167044465475</v>
       </c>
       <c r="T27" s="1">
         <v>4.7564085785623399E-2</v>
       </c>
+      <c r="V27">
+        <v>1.9</v>
+      </c>
+      <c r="W27" s="1">
+        <v>0.13548958029595701</v>
+      </c>
     </row>
-    <row r="28" spans="19:20" x14ac:dyDescent="0.25">
+    <row r="28" spans="19:23" x14ac:dyDescent="0.35">
       <c r="S28">
         <v>1.0142937182713132</v>
       </c>
       <c r="T28" s="1">
         <v>4.7594086855872998E-2</v>
       </c>
+      <c r="V28">
+        <v>1.9</v>
+      </c>
+      <c r="W28" s="1">
+        <v>0.13535257602050901</v>
+      </c>
     </row>
-    <row r="29" spans="19:20" x14ac:dyDescent="0.25">
+    <row r="29" spans="19:23" x14ac:dyDescent="0.35">
       <c r="S29">
         <v>1.0142937182713132</v>
       </c>
       <c r="T29" s="1">
         <v>4.7865832680007402E-2</v>
       </c>
+      <c r="V29">
+        <v>1.9</v>
+      </c>
+      <c r="W29" s="1">
+        <v>0.13521437182562601</v>
+      </c>
     </row>
-    <row r="30" spans="19:20" x14ac:dyDescent="0.25">
+    <row r="30" spans="19:23" x14ac:dyDescent="0.35">
       <c r="S30">
         <v>1.0142937182713132</v>
       </c>
       <c r="T30" s="1">
         <v>4.7946198533546001E-2</v>
       </c>
+      <c r="V30">
+        <v>1.9</v>
+      </c>
+      <c r="W30" s="1">
+        <v>0.13547579777680199</v>
+      </c>
     </row>
-    <row r="31" spans="19:20" x14ac:dyDescent="0.25">
+    <row r="31" spans="19:23" x14ac:dyDescent="0.35">
       <c r="S31">
         <v>1.0142937182713132</v>
       </c>
       <c r="T31" s="1">
         <v>4.7958321334516898E-2</v>
       </c>
+      <c r="V31">
+        <v>1.9</v>
+      </c>
+      <c r="W31" s="1">
+        <v>0.135355456711137</v>
+      </c>
     </row>
-    <row r="32" spans="19:20" x14ac:dyDescent="0.25">
+    <row r="32" spans="19:23" x14ac:dyDescent="0.35">
       <c r="S32">
         <v>1.0142937182713132</v>
       </c>
       <c r="T32" s="1">
         <v>4.7745472800668702E-2</v>
       </c>
+      <c r="V32">
+        <v>1.9</v>
+      </c>
+      <c r="W32" s="1">
+        <v>0.13562845171119001</v>
+      </c>
     </row>
-    <row r="33" spans="19:20" x14ac:dyDescent="0.25">
+    <row r="33" spans="19:23" x14ac:dyDescent="0.35">
       <c r="S33">
         <v>1.0142937182713132</v>
       </c>
       <c r="T33" s="1">
         <v>4.7683759372150601E-2</v>
       </c>
+      <c r="V33">
+        <v>1.9</v>
+      </c>
+      <c r="W33" s="1">
+        <v>0.135063967225622</v>
+      </c>
     </row>
-    <row r="34" spans="19:20" x14ac:dyDescent="0.25">
+    <row r="34" spans="19:23" x14ac:dyDescent="0.35">
       <c r="S34">
         <v>1.0142937182713132</v>
       </c>
       <c r="T34" s="1">
         <v>4.79771761493403E-2</v>
       </c>
+      <c r="V34">
+        <v>1.9</v>
+      </c>
+      <c r="W34" s="1">
+        <v>0.13488752919092301</v>
+      </c>
     </row>
-    <row r="35" spans="19:20" x14ac:dyDescent="0.25">
+    <row r="35" spans="19:23" x14ac:dyDescent="0.35">
       <c r="S35">
         <v>1.0142937182713132</v>
       </c>
       <c r="T35" s="1">
         <v>4.7459600367847798E-2</v>
       </c>
+      <c r="V35">
+        <v>1.9</v>
+      </c>
+      <c r="W35" s="1">
+        <v>0.13488940608340499</v>
+      </c>
     </row>
-    <row r="36" spans="19:20" x14ac:dyDescent="0.25">
+    <row r="36" spans="19:23" x14ac:dyDescent="0.35">
       <c r="S36">
         <v>1.0142937182713132</v>
       </c>
@@ -5563,7 +7240,7 @@
         <v>4.7677254085627299E-2</v>
       </c>
     </row>
-    <row r="37" spans="19:20" x14ac:dyDescent="0.25">
+    <row r="37" spans="19:23" x14ac:dyDescent="0.35">
       <c r="S37">
         <v>1.0142937182713132</v>
       </c>
@@ -5571,7 +7248,7 @@
         <v>4.79891735986843E-2</v>
       </c>
     </row>
-    <row r="38" spans="19:20" x14ac:dyDescent="0.25">
+    <row r="38" spans="19:23" x14ac:dyDescent="0.35">
       <c r="S38">
         <v>1.0142937182713132</v>
       </c>
@@ -5588,7 +7265,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C0E44BB-97B2-4005-A11E-A7B4189340B3}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>